<commit_message>
Improved GUI. Inplemented minimum window sizing and recolored to be more user friendly.
</commit_message>
<xml_diff>
--- a/employee_records.xlsx
+++ b/employee_records.xlsx
@@ -419,38 +419,40 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>employee_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>employee_name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>employee_department</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>employee_position</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>salary</t>
+          <t>employee_salary</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>hire_date</t>
+          <t>employee_hire_date</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1001</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -467,8 +469,10 @@
           <t>Structural Engineer</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>85000</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>85000</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -477,8 +481,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1002</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -495,8 +501,10 @@
           <t>CAD Designer</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>72000</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>72000</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -505,8 +513,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>1003</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1003</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -523,8 +533,10 @@
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>94000</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>94000</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>

</xml_diff>